<commit_message>
Add PostgreSQL database integration
</commit_message>
<xml_diff>
--- a/output/Product_Comparison_Report.xlsx
+++ b/output/Product_Comparison_Report.xlsx
@@ -1236,7 +1236,7 @@
       <c r="A17" s="3" t="inlineStr">
         <is>
           <t>'====================================================
-The review of the two product versions reveals significant modifications, with four parameters altered and one remaining unchanged. Notably, the plan description has been updated to extend the income benefit period from age 99 to 120, enhancing the product's appeal. Additionally, the maximum policy term and sum assured for the Point of Sale channel have been increased, reflecting a strategic shift towards more flexible offerings. The changes are primarily low to medium impact, indicating a focus on improving customer value without major operational disruptions.
+The review of the two versions of the insurance product reveals significant modifications, particularly in the Plan Description, Minimum/Maximum Maturity Age, and options available under the product. While the Premium Payment Frequency remains unchanged, the adjustments in the product's structure and benefits could enhance customer appeal and operational efficiency. The most notable change is the extension of the Income Period to age 120, which may attract a broader customer base. Overall, these modifications aim to improve the product's competitiveness in the market.
 ====================================================</t>
         </is>
       </c>
@@ -1259,10 +1259,10 @@
       <c r="A26" s="3" t="inlineStr">
         <is>
           <t>'====================================================
-1. Extension of the income benefit period from age 99 to 120.
-2. Increase in maximum policy term from 20 to 40 years for the Point of Sale channel.
-3. Increase in maximum sum assured from Rs. 25 lacs to Rs. 50 lacs for the Point of Sale channel.
-4. Modification of the maturity age for the Wealth Creation variant, changing the minimum age from 18 to 20.
+1. **Plan Description**: The Income Period has been extended from age 99 to age 120.
+2. **Minimum/Maximum Maturity Age**: Clarified age parameters for each variant, enhancing transparency.
+3. **Point of Sale Channel**: Increased maximum policy term from 20 to 40 years and maximum sum assured from Rs. 25 lacs to Rs. 50 lacs.
+4. **Options Available**: Enhanced flexibility in income installment options and the ability to change installment dates.
 ====================================================</t>
         </is>
       </c>
@@ -1288,11 +1288,11 @@
       <c r="A38" s="3" t="inlineStr">
         <is>
           <t>'====================================================
-- **Customer Impact**: The extended income benefit period and increased maximum sum assured enhance customer satisfaction and attract a broader demographic, particularly older clients seeking long-term financial security.
-- **Operations Impact**: The changes may require updates to operational processes, particularly in underwriting and claims management, to accommodate the new policy terms and conditions.
-- **Product Configuration Impact**: Adjustments in product configuration will be necessary to reflect the new parameters in the system, ensuring accurate policy issuance and management.
-- **UAT / Testing Impact**: User Acceptance Testing will need to be conducted to validate the changes in the product configuration, ensuring that all modifications function as intended before rollout.
-- **Compliance Impact**: The modifications must be reviewed for compliance with regulatory standards, particularly concerning the extended age limits and policy terms, to mitigate any legal risks.
+- **Customer Impact**: The extended Income Period and improved options may attract more customers seeking long-term financial security and flexibility in payment schedules.
+- **Operations Impact**: Adjustments in policy terms and conditions may require updates to operational processes and training for sales teams to ensure accurate communication with customers.
+- **Product Configuration Impact**: The changes necessitate updates to product configuration in the system to reflect new parameters and benefits accurately.
+- **UAT / Testing Impact**: Comprehensive testing will be required to validate the new configurations and ensure that all changes function as intended before launch.
+- **Compliance Impact**: The modifications must be reviewed to ensure compliance with regulatory standards, particularly concerning the extended age limits and payment options.
 ====================================================</t>
         </is>
       </c>
@@ -1323,11 +1323,11 @@
       <c r="A55" s="3" t="inlineStr">
         <is>
           <t>'====================================================
-1. Update product documentation to reflect the new parameters and ensure clarity for stakeholders.
-2. Coordinate with IT to implement necessary changes in the product configuration and ensure system readiness.
-3. Conduct a comprehensive UAT to validate all changes and ensure compliance with regulatory requirements.
-4. Prepare training materials for sales and customer service teams to familiarize them with the updated product features.
-5. Monitor customer feedback post-launch to assess the impact of changes and identify areas for further improvement.</t>
+1. Update product documentation to reflect all changes accurately.
+2. Conduct training sessions for sales and customer service teams on the new product features.
+3. Initiate a comprehensive UAT plan to test the new configurations and ensure system integrity.
+4. Review compliance implications with the legal team to ensure adherence to regulatory requirements.
+5. Develop a marketing strategy to promote the enhanced product features to potential customers.</t>
         </is>
       </c>
     </row>
@@ -1563,12 +1563,12 @@
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>The changes to the Income Period and premium wording significantly enhance the product's appeal and clarity, potentially leading to increased sales and customer satisfaction. However, careful communication and testing are necessary to mitigate any risks associated with misunderstanding the new terms.</t>
+          <t>The changes to the Income Period and premium wording significantly enhance the product's appeal and clarity, potentially leading to increased sales and customer satisfaction. However, careful communication and testing are necessary to mitigate any risks associated with customer understanding.</t>
         </is>
       </c>
       <c r="R3" s="3" t="inlineStr">
         <is>
-          <t>The increase in the Income Period from 99 years to 120 years allows policyholders to receive benefits for a longer duration, enhancing the product's attractiveness. The addition of 'prashil wanjari business analyst' may indicate a focus on improved analysis or customer service, potentially leading to better client engagement. The change in premium wording may simplify the understanding of premium options for customers, which could improve sales and customer satisfaction.</t>
+          <t>The increase in the Income Period from 99 years to 120 years allows policyholders to receive benefits for a longer duration, enhancing the product's attractiveness. The addition of 'prashil wanjari business analyst' may indicate a focus on improved analysis or customer service, potentially leading to better customer engagement. The change in premium wording may simplify the understanding of premium options for customers, which could improve sales and customer satisfaction.</t>
         </is>
       </c>
       <c r="S3" s="3" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="T3" s="3" t="inlineStr">
         <is>
-          <t>Conduct user acceptance testing to ensure that policyholders understand the changes and that the new wording is clear and accurate.</t>
+          <t>Conduct user acceptance testing to ensure that the changes are clearly communicated and understood by potential customers. Validate that all documentation reflects the new terms accurately.</t>
         </is>
       </c>
       <c r="U3" s="3" t="inlineStr">
@@ -1615,7 +1615,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Minimum/Maximum Maturity Age</t>
+          <t>Minimum/ Maximum Maturity Age</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
@@ -1644,17 +1644,17 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Maturity Age (lbd) in years Variant 1 - Lifelong Income Minimum 99 Maximum 99 Variant 2 - Second Income Minimum 35 Maximum 92 Variant 3 – Step-up Income Minimum 30 Maximum 89 Variant 4 – Extra Income Minimum 20 Single Life Policy: 75 Joint Life 74 Variant 5 – Wealth Creation Minimum 18 Maximum 60 Variant 6 - Assured Income Minimum 18 Maximum 60</t>
+          <t>Minimum 99, 35, 30, 20, 18, 18; Maximum 99, 92, 89; Single Life Policy: 75; Joint Life 74; Policy : 60</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>Maturity Age (lbd) in years Variant 1 - Lifelong Income Minimum 99 Maximum 99 Variant 2 - Second Income Minimum 35 Maximum 92 Variant 3 – Step-up Income Minimum 30 Maximum 89 Variant 4 – Extra Income Minimum 20 Single Life Policy: 75 Joint Life 74 Variant 5 – Wealth Creation Minimum 20 Policy : 60 Variant 6 - Assured Income Minimum 20</t>
+          <t>Minimum Maturity Age (lbd) in years: Variant 1 - Lifelong Income: 99, Variant 2 - Second Income: 35, Variant 3 – Step-up Income: 30, Variant 4 – Extra Income: 20, Variant 5 – Wealth Creation: 20, Variant 6 - Assured Income: 20. Maximum Maturity Age: Variant 1 - 99, Variant 2 - 92, Variant 3 - 89, Single Life Policy: 75, Joint Life: 74, Policy : 60</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>Modified: 18 → 20 for Variant 5 – Wealth Creation. Added: • 20 Policy : • 20. Removed: • 18 Maximum • 18 Maximum 60.</t>
+          <t>Minimum Maturity Age changed to include specific variants with associated ages. Maximum Maturity Age now specifies variants as well. Added detailed descriptions for each variant, while removing some previous values that were not specified in the new format.</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr"/>
@@ -1665,42 +1665,42 @@
       </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
-          <t>Ensure that all stakeholders are informed about the changes to avoid miscommunication with clients.</t>
+          <t>Ensure that all customer-facing materials are updated to reflect the new structure and that staff are trained on the changes.</t>
         </is>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>The adjustments to the maturity age and the addition of clarifying text are intended to enhance clarity but may require careful communication to ensure customer understanding and compliance.</t>
+          <t>The changes to the Minimum and Maximum Maturity Ages introduce a more detailed and variant-specific approach, which is expected to enhance product clarity and customer engagement, but requires careful communication to mitigate potential confusion.</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>The changes in the minimum maturity age for Variant 5 – Wealth Creation from 18 to 20 may affect the eligibility of younger clients seeking this policy. The addition of '20 Policy :' clarifies the maximum limit, which could influence customer understanding and decision-making.</t>
+          <t>The introduction of specific variants for Minimum and Maximum Maturity Ages allows for more tailored product offerings, potentially enhancing customer satisfaction and market competitiveness. This clarity in product structure may lead to improved sales and customer understanding of the options available.</t>
         </is>
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>Product Development, Marketing, Customer Service</t>
+          <t>Product Development, Marketing, Sales, Customer Support</t>
         </is>
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>Verify that all documentation reflects the new maturity age and that customer communications are updated to prevent confusion.</t>
+          <t>Conduct user acceptance testing to ensure that the new variant structure is clearly understood by customers and that all systems reflect the changes accurately.</t>
         </is>
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
-          <t>There is a risk of customer confusion regarding the new minimum age and the removal of the previous maximum age, potentially leading to misinterpretation of policy terms.</t>
+          <t>There is a risk of customer confusion if the new variant structure is not effectively communicated, as previous values have been removed and replaced with a more complex format.</t>
         </is>
       </c>
       <c r="V4" s="3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="W4" s="3" t="inlineStr">
         <is>
-          <t>Moderate; while the changes do not drastically alter the product, they may impact customer eligibility and understanding.</t>
+          <t>Critical, as it directly affects product offerings and customer engagement.</t>
         </is>
       </c>
     </row>
@@ -1875,32 +1875,32 @@
       </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>These changes are expected to enhance the product's market position and customer appeal.</t>
+          <t>The changes enhance the product offering but require careful monitoring of claims and financial implications.</t>
         </is>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>The modifications to the Maximum Policy Term and Maximum Sum Assured significantly enhance the product's attractiveness, potentially leading to increased sales and customer satisfaction while introducing new risks that need to be managed.</t>
+          <t>The modifications to the Maximum Policy Term and Maximum Sum Assured significantly enhance the product's appeal, potentially increasing market competitiveness and customer acquisition, while also necessitating careful risk management.</t>
         </is>
       </c>
       <c r="R6" s="3" t="inlineStr">
         <is>
-          <t>The increase in Maximum Policy Term allows customers to secure coverage for a longer duration, potentially enhancing customer satisfaction and retention. The higher Maximum Sum Assured increases the financial protection available to policyholders, making the product more attractive in a competitive market, which could lead to increased sales and market share.</t>
+          <t>The increase in Maximum Policy Term allows customers to secure coverage for a longer duration, potentially enhancing customer satisfaction and retention. The higher Maximum Sum Assured increases the financial protection available to policyholders, making the product more attractive in a competitive market.</t>
         </is>
       </c>
       <c r="S6" s="3" t="inlineStr">
         <is>
-          <t>Product Development, Sales, Marketing, Actuarial, Compliance</t>
+          <t>Product Development, Underwriting, Actuarial, Sales, Marketing</t>
         </is>
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>Conduct thorough testing to ensure that the new policy terms and sums assured are correctly implemented in the system and communicated to all stakeholders.</t>
+          <t>Conduct thorough testing to ensure that the new policy terms and sums assured are correctly implemented in the system and communicated to all relevant stakeholders.</t>
         </is>
       </c>
       <c r="U6" s="3" t="inlineStr">
         <is>
-          <t>There is a risk of increased claims liability due to the higher Maximum Sum Assured, which may impact the company's financial reserves if not managed properly.</t>
+          <t>There is a risk of increased claims liability due to the higher Maximum Sum Assured, which may impact the company's financial stability if not managed properly.</t>
         </is>
       </c>
       <c r="V6" s="3" t="inlineStr">
@@ -1910,7 +1910,7 @@
       </c>
       <c r="W6" s="3" t="inlineStr">
         <is>
-          <t>Critical, as it directly affects product competitiveness and customer appeal.</t>
+          <t>Critical</t>
         </is>
       </c>
     </row>
@@ -1961,17 +1961,17 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>a) Option to take the yearly Income Instalments in other instalment frequencies (only in Variants 1 to 4 &amp; 6) and Death Benefit Instalments (only in Variants 6) The default option in the product is annual Income Instalment. But the policyholder will have an option to take the same in other-than-yearly instalments. The Income Instalment frequency has to be chosen at inception. However, the policy holder will have an option to change the Income Instalment frequency once again during the policy term but before the income period starts. He can choose half-yearly, quarterly or monthly As per the Income Instalment frequency chosen by the policyholder, the instalments will be paid-out at the end of year, half-year, quarter or month from the end of the policy term, and at every subsequent half-year, quarter or month respectively. The half-yearly, quarterly or monthly installment will be arrived using the frequency factors given in above section “Income Instalments Frequency”, which will be applied on the yearly installment. The policyholder will not have the flexibility to change this option during income period Death Benefit Instalment: As on the date of death, and at every subsequent half-year, quarter or month respectively. b) Option to change the date of Income Instalment (only in Variants 1 to 4 &amp; 6) The Income Installment date has to be chosen at inception. However, the policy holder will have an option to change the Income Instalment date any time (no restrictions on number of changes) during the policy term but before the income period starts. Income Instalment date cannot be changed during the Income Period. The default option in the product is Income Instalment become due in arrear, i.e., one year after the end of policy term. But the policyholder will have an option to prepone the start of Income Installments by a maximum of 365 days, still within the Income Period. In any case the Income Installments (opted in any frequency) cannot be postpone from the due date. For Ex: - In case of yearly Income Instalments A policy is issued on 1st Jan 2021 with a policy term of 10 years. The default first yearly Income Installment will be payable on 1st Jan 2032. The policy holder will have an option to prepone the Income Installment date upto 1st Jan 2031 (Maximum of 365 days within the Income Period). In case of monthly Income Instalments A policy is issued on 1st Jan 2021 with a policy term of 10 years. The default first monthly Income Instalment will be payable on 1st Feb 2031. The policy holder will have an option to prepone the Income Instalment date upto 1st Jan 2031.</t>
+          <t>a) Option to take the yearly Income Instalments in other instalment frequencies (only in Variants 1 to 4 &amp; 6) and Death Benefit Instalments (only in Variants 6) The default option in the product is annual Income Instalment. But the policyholder will have an option to take the same in other-than-yearly instalments. The Income Instalment frequency has to be chosen at inception. However, the policy holder will have an option to change the Income Instalment frequency once again during the policy term but before the income period starts. He can choose half-yearly, quarterly or monthly. i) As per the Income Instalment frequency chosen by the policyholder, the instalments will be paid-out at the end of year, half-year, quarter or month from the end of the policy term, and at every subsequent half-year, quarter or month respectively. The half-yearly, quarterly or monthly installment will be arrived using the frequency factors given in above section “Income Instalments Frequency”, which will be applied on the yearly installment. The policyholder will not have the flexibility to change this option during income period. Death Benefit Instalment: As on the date of death, and at every subsequent half-year, quarter or month respectively. b) Option to change the date of Income Instalment (only in Variants 1 to 4 &amp; 6) The Income Installment date has to be chosen at inception. However, the policy holder will have an option to change the Income Instalment date any time (no restrictions on number of changes) during the policy term but before the income period starts. Income Instalment date cannot be changed during the Income Period. The default option in the product is Income Instalment become due in arrear, i.e., one year after the end of policy term. But the policyholder will have an option to prepone the start of Income Installments by a maximum of 365 days, still within the Income Period. In any case the Income Installments (opted in any frequency) cannot be postpone from the due date. For Ex: - In case of yearly Income Instalments A policy is issued on 1st Jan 2021 with a policy term of 10 years. The default first yearly Income Installment will be payable on 1st Jan 2032. The policy holder will have an option to prepone the Income Installment date upto 1st Jan 2031 (Maximum of 365 days within the Income Period). In case of monthly Income Instalments A policy is issued on 1st Jan 2021 with a policy term of 10 years. The default first monthly Income Instalment will be payable on 1st Feb 2031. The policy holder will have an option to prepone the Income Instalment date upto 1st Jan 2031.</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>a) Option to take the yearly Income Instalments in other instalment frequencies (only in Variants 1 to 4 &amp; 6) and Death Benefit Instalments (only in Variants 6) The default option in the product is annual Income Instalment. But the policyholder will have an option to take the same in other-than-yearly instalments. The Income Instalment frequency has to be chosen at inception. However, the policy holder will have an option to change the Income Instalment frequency once again during the policy term but before the income period starts. He can choose half-yearly, quarterly or monthly i) As per the Income Instalment frequency chosen by the policyholder, the instalments will be paid-out at the end of year, half-year, quarter or month from the end of the policy term, and at every subsequent half-year, quarter or month respectively. The half-yearly, quarterly or monthly installment will be arrived using the frequency factors given in above section “Income Instalments Frequency”, which will be applied on the yearly installment. The policyholder will not have the flexibility to change this option during income period Death Benefit Instalment: As on the date of death, and at every subsequent half-year, quarter or month respectively. b) Option to change the date of Income Instalment (only in Variants 1 to 4 &amp; 6) The Income Instalment date has to be chosen at inception. However, the policy holder will have an option to change the Income Instalment date any time (no restrictions on number of changes) during the policy term but before the income period starts. Income Instalment date cannot be changed during the Income Period. The default option in the product is Income Instalment become due in arrear, i.e., one year after the end of policy term. But the policyholder will have an option to prepone the start of Income Installments by a maximum of 365 days, still within the Income Period. In any case the Income Installments (opted in any frequency) cannot be postpone from the due date. For Ex: - In case of yearly Income Instalments A policy is issued on 1st Jan 2030 with a policy term of 10 years. The default first yearly Income Instalment will be payable on 1st Jan 2032. The policy holder will have an option to prepone the Income Instalment date upto 1st Jan 2040 (Maximum of 365 days within the Income Period). In case of monthly Income Instalments A policy is issued on 1st Jan 2024 with a policy term of 10 years. The default first monthly Income Instalment will be payable on 1st Feb 2045. The policy holder will have an option to prepone the Income Instalment date upto 1st Jan 2040.</t>
+          <t>a) Option to take the yearly Income Instalments in other instalment frequencies (only in Variants 1 to 4 &amp; 6) and Death Benefit Instalments (only in Variants 6) The default option in the product is annual Income Instalment. But the policyholder will have an option to take the same in other-than-yearly instalments. The Income Installment frequency has to be chosen at inception. However, the policy holder will have an option to change the Income Instalment frequency once again during the policy term but before the income period starts. He can choose half-yearly, quarterly or monthly. i) As per the Income Instalment frequency chosen by the policyholder, the instalments will be paid-out at the end of year, half-year, quarter or month from the end of the policy term, and at every subsequent half-year, quarter or month respectively. The half-yearly, quarterly or monthly installment will be arrived using the frequency factors given in above section “Income Instalments Frequency”, which will be applied on the yearly installment. The policyholder will not have the flexibility to change this option during income period. Death Benefit Instalment: As on the date of death, and at every subsequent half-year, quarter or month respectively. b) Option to change the date of Income Instalment (only in Variants 1 to 4 &amp; 6) The Income Installment date has to be chosen at inception. However, the policy holder will have an option to change the Income Instalment date any time (no restrictions on number of changes) during the policy term but before the income period starts. Income Instalment date cannot be changed during the Income Period. The default option in the product is Income Instalment become due in arrear, i.e., one year after the end of policy term. But the policyholder will have an option to prepone the start of Income Installments by a maximum of 365 days, still within the Income Period. In any case the Income Installments (opted in any frequency) cannot be postpone from the due date. For Ex: - In case of yearly Income Instalments A policy is issued on 1st Jan 2030 with a policy term of 10 years. The default first yearly Income Installment will be payable on 1st Jan 2032. The policy holder will have an option to prepone the Income Installment date upto 1st Jan 2040 (Maximum of 365 days within the Income Period). In case of monthly Income Instalments A policy is issued on 1st Jan 2024 with a policy term of 10 years. The default first monthly Income Instalment will be payable on 1st Feb 2045. The policy holder will have an option to prepone the Income Instalment date upto 1st Jan 2040.</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>Modified: 2021 → 2030; Modified: 2031 → 2040; Modified: 2021 → 2024; Modified: 2031 → 2045; Modified: 2031 → 2040; Added: i); Instalment; 2030; Instalment; Instalment; 2040; 2024; 2045; 2040; Removed: Installment; 2021; Installment; Installment; 2031; 2021; 2031; 2031.</t>
+          <t>Modified: 2021 → 2030; Modified: 2031 → 2040; Modified: 2021 → 2024; Modified: 2031 → 2045; Modified: 2031 → 2040; Added: Installment, 2030, 2040, 2024, 2045; Removed: Instalment, 2021, 2031, 2021, 2031, 2031.</t>
         </is>
       </c>
       <c r="N7" s="3" t="inlineStr"/>
@@ -1982,32 +1982,32 @@
       </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>Ensure all customer-facing materials are updated to reflect the new terms and that staff are trained on the changes to avoid misinformation.</t>
+          <t>Ensure that all customer-facing materials are updated to reflect the new dates and clarify any potential confusion.</t>
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>The modifications to the Income Instalment dates and options enhance flexibility for policyholders but require careful management to mitigate risks associated with customer confusion and operational adjustments. The changes are critical to maintaining customer satisfaction and operational efficiency.</t>
+          <t>The changes to the installment dates and the introduction of new years for policy issuance are significant and require careful management to ensure customer understanding and satisfaction. The potential for confusion necessitates a proactive communication strategy.</t>
         </is>
       </c>
       <c r="R7" s="3" t="inlineStr">
         <is>
-          <t>The changes in dates for the Income Instalments indicate a shift in the policy's timeline, potentially affecting cash flow projections and financial planning for policyholders. The ability to prepone instalment dates may enhance customer satisfaction by providing more flexibility, but it also requires careful management of cash reserves. The removal of certain years suggests a refinement in the product offering, which could streamline operations but may also necessitate updates in training and communication for affected teams.</t>
+          <t>The changes in dates for policy issuance and installment payments may affect the timing of cash flows for policyholders. The new dates allow for a longer period before the first installment is due, which could impact customer expectations and financial planning. Additionally, the removal of certain years may lead to confusion if not communicated effectively, potentially affecting customer satisfaction and retention.</t>
         </is>
       </c>
       <c r="S7" s="3" t="inlineStr">
         <is>
-          <t>Product Development, Customer Service, Compliance, IT</t>
+          <t>Product Management, Customer Service, Marketing, Compliance</t>
         </is>
       </c>
       <c r="T7" s="3" t="inlineStr">
         <is>
-          <t>Conduct thorough testing of the updated policy terms in the system to ensure accurate processing of instalment dates and options. User acceptance testing with customer service representatives is recommended to validate understanding and communication of changes.</t>
+          <t>Conduct thorough testing of the policy issuance and payment schedule systems to ensure that the new dates are correctly implemented and communicated to customers.</t>
         </is>
       </c>
       <c r="U7" s="3" t="inlineStr">
         <is>
-          <t>There is a risk of confusion among policyholders regarding the new dates and options for Income Instalments, which could lead to dissatisfaction or errors in payment processing. Additionally, the changes may require updates to systems and documentation, posing a risk of implementation errors.</t>
+          <t>There is a risk of customer dissatisfaction due to potential confusion over the new installment dates. If not properly communicated, policyholders may misinterpret their payment schedules, leading to missed payments or complaints.</t>
         </is>
       </c>
       <c r="V7" s="3" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Maturity Age (lbd) in years Variant 1 - Lifelong Income Minimum 99 Maximum 99 Variant 2 - Second Income Minimum 35 Maximum 92 Variant 3 – Step-up Income Minimum 30 Maximum 89 Variant 4 – Extra Income Minimum 20 Single Life Policy: 75 Joint Life 74 Variant 5 – Wealth Creation Minimum 18 Maximum 60 Variant 6 - Assured Income Minimum 18 Maximum 60</t>
+          <t>Minimum 99, 35, 30, 20, 18, 18; Maximum 99, 92, 89; Single Life Policy: 75; Joint Life 74; Policy : 60</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
@@ -2457,7 +2457,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>a) Option to take the yearly Income Instalments in other instalment frequencies (only in Variants 1 to 4 &amp; 6) and Death Benefit Instalments (only in Variants 6) The default option in the product is annual Income Instalment. But the policyholder will have an option to take the same in other-than-yearly instalments. The Income Instalment frequency has to be chosen at inception. However, the policy holder will have an option to change the Income Instalment frequency once again during the policy term but before the income period starts. He can choose half-yearly, quarterly or monthly As per the Income Instalment frequency chosen by the policyholder, the instalments will be paid-out at the end of year, half-year, quarter or month from the end of the policy term, and at every subsequent half-year, quarter or month respectively. The half-yearly, quarterly or monthly installment will be arrived using the frequency factors given in above section “Income Instalments Frequency”, which will be applied on the yearly installment. The policyholder will not have the flexibility to change this option during income period Death Benefit Instalment: As on the date of death, and at every subsequent half-year, quarter or month respectively. b) Option to change the date of Income Instalment (only in Variants 1 to 4 &amp; 6) The Income Installment date has to be chosen at inception. However, the policy holder will have an option to change the Income Instalment date any time (no restrictions on number of changes) during the policy term but before the income period starts. Income Instalment date cannot be changed during the Income Period. The default option in the product is Income Instalment become due in arrear, i.e., one year after the end of policy term. But the policyholder will have an option to prepone the start of Income Installments by a maximum of 365 days, still within the Income Period. In any case the Income Installments (opted in any frequency) cannot be postpone from the due date. For Ex: - In case of yearly Income Instalments A policy is issued on 1st Jan 2021 with a policy term of 10 years. The default first yearly Income Installment will be payable on 1st Jan 2032. The policy holder will have an option to prepone the Income Installment date upto 1st Jan 2031 (Maximum of 365 days within the Income Period). In case of monthly Income Instalments A policy is issued on 1st Jan 2021 with a policy term of 10 years. The default first monthly Income Instalment will be payable on 1st Feb 2031. The policy holder will have an option to prepone the Income Instalment date upto 1st Jan 2031.</t>
+          <t>a) Option to take the yearly Income Instalments in other instalment frequencies (only in Variants 1 to 4 &amp; 6) and Death Benefit Instalments (only in Variants 6) The default option in the product is annual Income Instalment. But the policyholder will have an option to take the same in other-than-yearly instalments. The Income Instalment frequency has to be chosen at inception. However, the policy holder will have an option to change the Income Instalment frequency once again during the policy term but before the income period starts. He can choose half-yearly, quarterly or monthly. i) As per the Income Instalment frequency chosen by the policyholder, the instalments will be paid-out at the end of year, half-year, quarter or month from the end of the policy term, and at every subsequent half-year, quarter or month respectively. The half-yearly, quarterly or monthly installment will be arrived using the frequency factors given in above section “Income Instalments Frequency”, which will be applied on the yearly installment. The policyholder will not have the flexibility to change this option during income period. Death Benefit Instalment: As on the date of death, and at every subsequent half-year, quarter or month respectively. b) Option to change the date of Income Instalment (only in Variants 1 to 4 &amp; 6) The Income Installment date has to be chosen at inception. However, the policy holder will have an option to change the Income Instalment date any time (no restrictions on number of changes) during the policy term but before the income period starts. Income Instalment date cannot be changed during the Income Period. The default option in the product is Income Instalment become due in arrear, i.e., one year after the end of policy term. But the policyholder will have an option to prepone the start of Income Installments by a maximum of 365 days, still within the Income Period. In any case the Income Installments (opted in any frequency) cannot be postpone from the due date. For Ex: - In case of yearly Income Instalments A policy is issued on 1st Jan 2021 with a policy term of 10 years. The default first yearly Income Installment will be payable on 1st Jan 2032. The policy holder will have an option to prepone the Income Installment date upto 1st Jan 2031 (Maximum of 365 days within the Income Period). In case of monthly Income Instalments A policy is issued on 1st Jan 2021 with a policy term of 10 years. The default first monthly Income Instalment will be payable on 1st Feb 2031. The policy holder will have an option to prepone the Income Instalment date upto 1st Jan 2031.</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr"/>
@@ -2604,12 +2604,12 @@
     <row r="11" ht="34" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Minimum/Maximum Maturity Age</t>
+          <t>Minimum/ Maximum Maturity Age</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Maturity Age (lbd) in years Variant 1 - Lifelong Income Minimum 99 Maximum 99 Variant 2 - Second Income Minimum 35 Maximum 92 Variant 3 – Step-up Income Minimum 30 Maximum 89 Variant 4 – Extra Income Minimum 20 Single Life Policy: 75 Joint Life 74 Variant 5 – Wealth Creation Minimum 20 Policy : 60 Variant 6 - Assured Income Minimum 20</t>
+          <t>Minimum Maturity Age (lbd) in years: Variant 1 - Lifelong Income: 99, Variant 2 - Second Income: 35, Variant 3 – Step-up Income: 30, Variant 4 – Extra Income: 20, Variant 5 – Wealth Creation: 20, Variant 6 - Assured Income: 20. Maximum Maturity Age: Variant 1 - 99, Variant 2 - 92, Variant 3 - 89, Single Life Policy: 75, Joint Life: 74, Policy : 60</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
@@ -2681,7 +2681,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>a) Option to take the yearly Income Instalments in other instalment frequencies (only in Variants 1 to 4 &amp; 6) and Death Benefit Instalments (only in Variants 6) The default option in the product is annual Income Instalment. But the policyholder will have an option to take the same in other-than-yearly instalments. The Income Instalment frequency has to be chosen at inception. However, the policy holder will have an option to change the Income Instalment frequency once again during the policy term but before the income period starts. He can choose half-yearly, quarterly or monthly i) As per the Income Instalment frequency chosen by the policyholder, the instalments will be paid-out at the end of year, half-year, quarter or month from the end of the policy term, and at every subsequent half-year, quarter or month respectively. The half-yearly, quarterly or monthly installment will be arrived using the frequency factors given in above section “Income Instalments Frequency”, which will be applied on the yearly installment. The policyholder will not have the flexibility to change this option during income period Death Benefit Instalment: As on the date of death, and at every subsequent half-year, quarter or month respectively. b) Option to change the date of Income Instalment (only in Variants 1 to 4 &amp; 6) The Income Instalment date has to be chosen at inception. However, the policy holder will have an option to change the Income Instalment date any time (no restrictions on number of changes) during the policy term but before the income period starts. Income Instalment date cannot be changed during the Income Period. The default option in the product is Income Instalment become due in arrear, i.e., one year after the end of policy term. But the policyholder will have an option to prepone the start of Income Installments by a maximum of 365 days, still within the Income Period. In any case the Income Installments (opted in any frequency) cannot be postpone from the due date. For Ex: - In case of yearly Income Instalments A policy is issued on 1st Jan 2030 with a policy term of 10 years. The default first yearly Income Instalment will be payable on 1st Jan 2032. The policy holder will have an option to prepone the Income Instalment date upto 1st Jan 2040 (Maximum of 365 days within the Income Period). In case of monthly Income Instalments A policy is issued on 1st Jan 2024 with a policy term of 10 years. The default first monthly Income Instalment will be payable on 1st Feb 2045. The policy holder will have an option to prepone the Income Instalment date upto 1st Jan 2040.</t>
+          <t>a) Option to take the yearly Income Instalments in other instalment frequencies (only in Variants 1 to 4 &amp; 6) and Death Benefit Instalments (only in Variants 6) The default option in the product is annual Income Instalment. But the policyholder will have an option to take the same in other-than-yearly instalments. The Income Installment frequency has to be chosen at inception. However, the policy holder will have an option to change the Income Instalment frequency once again during the policy term but before the income period starts. He can choose half-yearly, quarterly or monthly. i) As per the Income Instalment frequency chosen by the policyholder, the instalments will be paid-out at the end of year, half-year, quarter or month from the end of the policy term, and at every subsequent half-year, quarter or month respectively. The half-yearly, quarterly or monthly installment will be arrived using the frequency factors given in above section “Income Instalments Frequency”, which will be applied on the yearly installment. The policyholder will not have the flexibility to change this option during income period. Death Benefit Instalment: As on the date of death, and at every subsequent half-year, quarter or month respectively. b) Option to change the date of Income Instalment (only in Variants 1 to 4 &amp; 6) The Income Installment date has to be chosen at inception. However, the policy holder will have an option to change the Income Instalment date any time (no restrictions on number of changes) during the policy term but before the income period starts. Income Instalment date cannot be changed during the Income Period. The default option in the product is Income Instalment become due in arrear, i.e., one year after the end of policy term. But the policyholder will have an option to prepone the start of Income Installments by a maximum of 365 days, still within the Income Period. In any case the Income Installments (opted in any frequency) cannot be postpone from the due date. For Ex: - In case of yearly Income Instalments A policy is issued on 1st Jan 2030 with a policy term of 10 years. The default first yearly Income Installment will be payable on 1st Jan 2032. The policy holder will have an option to prepone the Income Installment date upto 1st Jan 2040 (Maximum of 365 days within the Income Period). In case of monthly Income Instalments A policy is issued on 1st Jan 2024 with a policy term of 10 years. The default first monthly Income Instalment will be payable on 1st Feb 2045. The policy holder will have an option to prepone the Income Instalment date upto 1st Jan 2040.</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr"/>
@@ -2744,30 +2744,30 @@
           <t>'====================================================
 EXECUTIVE SUMMARY
 ====================================================
-The review of the two product versions reveals significant modifications, with four parameters altered and one remaining unchanged. Notably, the plan description has been updated to extend the income benefit period from age 99 to 120, enhancing the product's appeal. Additionally, the maximum policy term and sum assured for the Point of Sale channel have been increased, reflecting a strategic shift towards more flexible offerings. The changes are primarily low to medium impact, indicating a focus on improving customer value without major operational disruptions.
+The review of the two versions of the insurance product reveals significant modifications, particularly in the Plan Description, Minimum/Maximum Maturity Age, and options available under the product. While the Premium Payment Frequency remains unchanged, the adjustments in the product's structure and benefits could enhance customer appeal and operational efficiency. The most notable change is the extension of the Income Period to age 120, which may attract a broader customer base. Overall, these modifications aim to improve the product's competitiveness in the market.
 ====================================================
 KEY BUSINESS CHANGES
 ====================================================
-1. Extension of the income benefit period from age 99 to 120.
-2. Increase in maximum policy term from 20 to 40 years for the Point of Sale channel.
-3. Increase in maximum sum assured from Rs. 25 lacs to Rs. 50 lacs for the Point of Sale channel.
-4. Modification of the maturity age for the Wealth Creation variant, changing the minimum age from 18 to 20.
+1. **Plan Description**: The Income Period has been extended from age 99 to age 120.
+2. **Minimum/Maximum Maturity Age**: Clarified age parameters for each variant, enhancing transparency.
+3. **Point of Sale Channel**: Increased maximum policy term from 20 to 40 years and maximum sum assured from Rs. 25 lacs to Rs. 50 lacs.
+4. **Options Available**: Enhanced flexibility in income installment options and the ability to change installment dates.
 ====================================================
 BUSINESS IMPACT
 ====================================================
-- **Customer Impact**: The extended income benefit period and increased maximum sum assured enhance customer satisfaction and attract a broader demographic, particularly older clients seeking long-term financial security.
-- **Operations Impact**: The changes may require updates to operational processes, particularly in underwriting and claims management, to accommodate the new policy terms and conditions.
-- **Product Configuration Impact**: Adjustments in product configuration will be necessary to reflect the new parameters in the system, ensuring accurate policy issuance and management.
-- **UAT / Testing Impact**: User Acceptance Testing will need to be conducted to validate the changes in the product configuration, ensuring that all modifications function as intended before rollout.
-- **Compliance Impact**: The modifications must be reviewed for compliance with regulatory standards, particularly concerning the extended age limits and policy terms, to mitigate any legal risks.
+- **Customer Impact**: The extended Income Period and improved options may attract more customers seeking long-term financial security and flexibility in payment schedules.
+- **Operations Impact**: Adjustments in policy terms and conditions may require updates to operational processes and training for sales teams to ensure accurate communication with customers.
+- **Product Configuration Impact**: The changes necessitate updates to product configuration in the system to reflect new parameters and benefits accurately.
+- **UAT / Testing Impact**: Comprehensive testing will be required to validate the new configurations and ensure that all changes function as intended before launch.
+- **Compliance Impact**: The modifications must be reviewed to ensure compliance with regulatory standards, particularly concerning the extended age limits and payment options.
 ====================================================
 RECOMMENDED ACTIONS
 ====================================================
-1. Update product documentation to reflect the new parameters and ensure clarity for stakeholders.
-2. Coordinate with IT to implement necessary changes in the product configuration and ensure system readiness.
-3. Conduct a comprehensive UAT to validate all changes and ensure compliance with regulatory requirements.
-4. Prepare training materials for sales and customer service teams to familiarize them with the updated product features.
-5. Monitor customer feedback post-launch to assess the impact of changes and identify areas for further improvement.</t>
+1. Update product documentation to reflect all changes accurately.
+2. Conduct training sessions for sales and customer service teams on the new product features.
+3. Initiate a comprehensive UAT plan to test the new configurations and ensure system integrity.
+4. Review compliance implications with the legal team to ensure adherence to regulatory requirements.
+5. Develop a marketing strategy to promote the enhanced product features to potential customers.</t>
         </is>
       </c>
     </row>

</xml_diff>